<commit_message>
add 2026 branch and some new instructions
</commit_message>
<xml_diff>
--- a/corpus/aux/EcoCorMetadata.xlsx
+++ b/corpus/aux/EcoCorMetadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniilskorinkin/ACTIVITIES/DH NETZWERK and more/Climate DH/EcoCor/preparation stage/Making TEI/Repo/ecocor/corpus/aux/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniilskorinkin/ACTIVITIES/DH_NETZWERK/EcoCor_and_Climate DH/EcoCor/EcoCor2026/TEI conversion/ecocor/corpus/aux/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B7380C-6640-7641-B383-E2CB2FA624A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080D43A5-F8B8-264D-9755-47FE490F22A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="392">
   <si>
     <t>Autor*in</t>
   </si>
@@ -1184,13 +1184,25 @@
   </si>
   <si>
     <t>F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">David Friedrich Weinland </t>
+  </si>
+  <si>
+    <t>Rulaman</t>
+  </si>
+  <si>
+    <t>https://www.wikidata.org/wiki/Q1615214</t>
+  </si>
+  <si>
+    <t>EzProse_Example David_Friedrich_Weinland_-_Rulaman_(1878)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1203,6 +1215,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1248,19 +1268,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1561,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P69"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
@@ -4308,7 +4334,7 @@
       <c r="G69" t="s">
         <v>375</v>
       </c>
-      <c r="H69" t="s">
+      <c r="H69" s="3" t="s">
         <v>382</v>
       </c>
       <c r="I69" t="s">
@@ -4327,7 +4353,40 @@
         <v>386</v>
       </c>
     </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A70" s="4">
+        <v>74</v>
+      </c>
+      <c r="B70" t="s">
+        <v>388</v>
+      </c>
+      <c r="C70" t="s">
+        <v>389</v>
+      </c>
+      <c r="E70">
+        <v>1878</v>
+      </c>
+      <c r="F70" t="s">
+        <v>185</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K70" t="s">
+        <v>391</v>
+      </c>
+      <c r="O70">
+        <v>1878</v>
+      </c>
+      <c r="P70" t="s">
+        <v>386</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H69" r:id="rId1" xr:uid="{0FE63742-4B58-184A-83EF-25BBA056EFC0}"/>
+    <hyperlink ref="H70" r:id="rId2" xr:uid="{8501E2B3-F9FF-F74C-BEEB-A8F1D0B2E396}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>